<commit_message>
Atleast the ghost moves IG
</commit_message>
<xml_diff>
--- a/Data/level1.xlsx
+++ b/Data/level1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Dae assignments\2024-2025\Prog4\Prog4-Exam-MsPacMan\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{253797EF-FC82-4BB1-A1C9-EC7C92E2736C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8FE4FA2-5695-4F0D-942D-B2804755E7CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3E7511AE-F3C7-412D-A4F9-E82611F2F07B}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="16">
   <si>
     <t>7 90</t>
   </si>
@@ -53,6 +53,21 @@
   </si>
   <si>
     <t>2 90</t>
+  </si>
+  <si>
+    <t>Inky</t>
+  </si>
+  <si>
+    <t>Pinky</t>
+  </si>
+  <si>
+    <t>Clyde</t>
+  </si>
+  <si>
+    <t>Blinky</t>
+  </si>
+  <si>
+    <t>FA</t>
   </si>
 </sst>
 </file>
@@ -195,7 +210,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -378,6 +393,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -542,7 +563,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -550,6 +571,7 @@
     <xf numFmtId="3" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -599,14 +621,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="0"/>
+          <bgColor rgb="FFFFFF99"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFF99"/>
+          <bgColor theme="0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1875,9 +1897,15 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
+      <c r="M12" t="s">
+        <v>14</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
@@ -2054,12 +2082,15 @@
       <c r="K15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
+      <c r="L15" t="s">
+        <v>11</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="P15" t="s">
+        <v>13</v>
+      </c>
       <c r="R15" s="2">
         <v>1270</v>
       </c>
@@ -3333,12 +3364,12 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:AB31">
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="P">
+  <conditionalFormatting sqref="A15:P15 R15:AB15 A16:AB31 A1:AB14">
+    <cfRule type="containsBlanks" dxfId="1" priority="1">
+      <formula>LEN(TRIM(A1))=0</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="P">
       <formula>NOT(ISERROR(SEARCH("P",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(A1))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>